<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@8aab88593620927cf49b9aa390d655c1178a068e 🚀
</commit_message>
<xml_diff>
--- a/StructureDefinition-PractitionerRole.xlsx
+++ b/StructureDefinition-PractitionerRole.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-07-26T10:53:24+00:00</t>
+    <t>2024-07-26T11:32:38+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -623,7 +623,7 @@
     <t>Roles which this practitioner may perform</t>
   </si>
   <si>
-    <t>Roles which this practitioner is authorized to perform for the organization.</t>
+    <t>Zie [ConceptMap-epic-rolcode](ConceptMap-epic-rolcode.html)</t>
   </si>
   <si>
     <t>A person may have more than one role. Note: in earlier versions of this profile there used to be an association with the HCIM element NL-CM:17.1.5 HealthProfessionalRole. This mapping was semantically incorrect. The HCIM element is a property of the association of PractitionerRole to some healthcare act. In a number of FHIR Resources the association is implicit from the semantics of the resource element like in `Observation.performer`. In others you can make this explicit like `Encounter.participant.type`, `CareTeam.participant.role` and `Procedure.performer.role`. Please refer to the relevant profiles on those resources for associations with HCIM NL-CM:17.1.5 HealthProfessionalRole.</t>
@@ -3658,7 +3658,7 @@
         <v>85</v>
       </c>
       <c r="H16" t="s" s="2">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="I16" t="s" s="2">
         <v>83</v>

</xml_diff>